<commit_message>
Agregar calculos de desbalance trifasico
</commit_message>
<xml_diff>
--- a/datos/motores.xlsx
+++ b/datos/motores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Electrical_Engineering\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2C4CE6-9B19-4BEA-81B8-C0B872F6BB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4BE601-45EC-44E9-B4C3-017CC4DDDD78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CF66B361-FEBB-41C8-94E9-5375418F99E3}"/>
   </bookViews>
@@ -34,54 +34,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>TAG</t>
   </si>
   <si>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>VOLTAJE</t>
+  </si>
+  <si>
+    <t>FP</t>
+  </si>
+  <si>
+    <t>EFICIENCIA</t>
+  </si>
+  <si>
+    <t>M-001</t>
+  </si>
+  <si>
+    <t>M-002</t>
+  </si>
+  <si>
+    <t>M-003</t>
+  </si>
+  <si>
+    <t>CORRIENTE_PLACA_A</t>
+  </si>
+  <si>
     <t>DESCRIPCION</t>
   </si>
   <si>
-    <t>HP</t>
-  </si>
-  <si>
-    <t>VOLTAJE</t>
-  </si>
-  <si>
-    <t>FP</t>
-  </si>
-  <si>
-    <t>EFICIENCIA</t>
-  </si>
-  <si>
-    <t>M-001</t>
+    <t>CORRIENTE_L1_A</t>
+  </si>
+  <si>
+    <t>CORRIENTE_L2_A</t>
+  </si>
+  <si>
+    <t>CORRIENTE_L3_A</t>
+  </si>
+  <si>
+    <t>VOLTAJE_L1_L2_V</t>
+  </si>
+  <si>
+    <t>VOLTAJE_L2_L3_V</t>
+  </si>
+  <si>
+    <t>VOLTAJE_L3_L1_V</t>
+  </si>
+  <si>
+    <t>ESTADO</t>
   </si>
   <si>
     <t>Bomba de agua</t>
   </si>
   <si>
-    <t>M-002</t>
+    <t>Operando</t>
   </si>
   <si>
     <t>Ventilador</t>
   </si>
   <si>
-    <t>M-003</t>
-  </si>
-  <si>
     <t>Bomba condensado</t>
-  </si>
-  <si>
-    <t>CORRIENTE_PLACA_A</t>
-  </si>
-  <si>
-    <t>CORRIENTE_MEDIDA_A</t>
-  </si>
-  <si>
-    <t>ESTADO</t>
-  </si>
-  <si>
-    <t>Operando</t>
   </si>
 </sst>
 </file>
@@ -130,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -138,15 +153,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -465,135 +471,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F3007C-4CCE-4FA5-A545-AD73C08BCFA6}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.08984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.6328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" style="7" customWidth="1"/>
-    <col min="8" max="8" width="12.6328125" style="7" customWidth="1"/>
-    <col min="9" max="9" width="9.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" style="2"/>
+    <col min="3" max="3" width="4.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.26953125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="18.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="42" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>14</v>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3">
+        <v>125</v>
+      </c>
+      <c r="D2" s="3">
+        <v>480</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0.94</v>
+      </c>
+      <c r="G2" s="3">
+        <v>140</v>
+      </c>
+      <c r="H2" s="3">
+        <v>118</v>
+      </c>
+      <c r="I2" s="3">
+        <v>120</v>
+      </c>
+      <c r="J2" s="3">
+        <v>123</v>
+      </c>
+      <c r="K2" s="3">
+        <v>478</v>
+      </c>
+      <c r="L2" s="3">
+        <v>481</v>
+      </c>
+      <c r="M2" s="3">
+        <v>479</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3">
+        <v>75</v>
+      </c>
+      <c r="D3" s="3">
+        <v>480</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.9</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.93</v>
+      </c>
+      <c r="G3" s="3">
+        <v>82</v>
+      </c>
+      <c r="H3" s="3">
+        <v>74</v>
+      </c>
+      <c r="I3" s="3">
+        <v>76</v>
+      </c>
+      <c r="J3" s="3">
+        <v>79</v>
+      </c>
+      <c r="K3" s="3">
+        <v>477</v>
+      </c>
+      <c r="L3" s="3">
+        <v>480</v>
+      </c>
+      <c r="M3" s="3">
+        <v>482</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="5">
-        <v>125</v>
-      </c>
-      <c r="D2" s="5">
+      <c r="B4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3">
+        <v>30</v>
+      </c>
+      <c r="D4" s="3">
         <v>480</v>
       </c>
-      <c r="E2" s="6">
-        <v>0.88</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0.94</v>
-      </c>
-      <c r="G2" s="5">
-        <v>140</v>
-      </c>
-      <c r="H2" s="5">
-        <v>120</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5">
-        <v>75</v>
-      </c>
-      <c r="D3" s="5">
-        <v>480</v>
-      </c>
-      <c r="E3" s="6">
-        <v>0.9</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0.93</v>
-      </c>
-      <c r="G3" s="5">
-        <v>82</v>
-      </c>
-      <c r="H3" s="5">
-        <v>76</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="5">
-        <v>30</v>
-      </c>
-      <c r="D4" s="5">
-        <v>480</v>
-      </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>0.87</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.91</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="3">
         <v>35</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="3">
+        <v>31</v>
+      </c>
+      <c r="I4" s="3">
         <v>32</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>15</v>
+      <c r="J4" s="3">
+        <v>33</v>
+      </c>
+      <c r="K4" s="3">
+        <v>479</v>
+      </c>
+      <c r="L4" s="3">
+        <v>478</v>
+      </c>
+      <c r="M4" s="3">
+        <v>481</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>